<commit_message>
Update evaluation form and Excel template per user feedback
Word document changes:
- Moved 'Does Not Meet Expectations' checkbox to its own line
- Removed Comments sections from rating criteria (I-IV)
- Removed horizontal line before signature section
- Removed Notes fields from Additional Information sections
- Changed font to Times New Roman

Excel template changes:
- Added second date range column for each course
- Supports instructors who teach the same course twice per year
- Updated examples and instructions

https://claude.ai/code/session_019joi3KhwMT9HyLdFbSuVpw
</commit_message>
<xml_diff>
--- a/PTL_Evaluation_Data_Template.xlsx
+++ b/PTL_Evaluation_Data_Template.xlsx
@@ -67,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -78,6 +78,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment indent="4"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -444,24 +447,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Faculty First Name</t>
@@ -484,40 +491,60 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Course 1 Dates</t>
+          <t>Course 1 Dates (1st)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Course 1 Dates (2nd)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Course 2</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Course 2 Dates</t>
-        </is>
-      </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Course 2 Dates (1st)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Course 2 Dates (2nd)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Course 3</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Course 3 Dates</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Course 3 Dates (1st)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Course 3 Dates (2nd)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Course 4</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Course 4 Dates</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Course 4 Dates (1st)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Course 4 Dates (2nd)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>AACSB Status</t>
         </is>
@@ -549,21 +576,25 @@
           <t>1/12/26 - 2/15/26</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>ACCT 202</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>2/16/26 - 4/15/26</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Scholarly Practitioner</t>
         </is>
@@ -597,29 +628,87 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>8/15/26 - 10/30/26</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>MGMT 405</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>1/12/26 - 3/01/26</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>MGMT 410</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>3/15/26 - 5/01/26</t>
-        </is>
-      </c>
+      <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>Instructional Practitioner</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Robert</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Johnson</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>FIN 301</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>1/12/26 - 3/01/26</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>3/15/26 - 5/15/26</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>FIN 301</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>8/15/26 - 10/30/26</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>11/01/26 - 12/15/26</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Practice Academic</t>
         </is>
       </c>
     </row>
@@ -634,10 +723,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="85" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -688,81 +777,126 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>• Course Dates: Date range for each course (e.g., 1/12/26 - 2/15/26)</t>
+          <t>• Course Dates (1st): First date range for the course (e.g., 1/12/26 - 2/15/26)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>• Course Dates (2nd): Second date range if the same course is taught twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>• AACSB Status: Faculty qualification status</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Notes:</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>• Leave Course/Date fields blank if instructor teaches fewer than 4 courses</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>• If instructor teaches more than 4 courses, add additional columns as needed</t>
+          <t>• If an instructor teaches the SAME course twice in one year, enter both date ranges</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>• The automation script will merge First Name + Last Name and combine all courses</t>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Example: MGMT 301 taught in Spring AND Fall - enter dates in (1st) and (2nd) columns</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>• Leave Course/Date fields blank if instructor teaches fewer courses</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Common AACSB Status Values:</t>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>• If instructor teaches more than 4 different courses, add additional columns as needed</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>• Scholarly Academic (SA)</t>
+          <t>• The automation script will merge First Name + Last Name and combine all courses with dates</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>• Practice Academic (PA)</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>• Scholarly Practitioner (SP)</t>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Example Output Format:</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>• Single offering: ACCT 201 (1/12/26 - 2/15/26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>• Two offerings: MGMT 301 (1/12/26 - 3/01/26, 8/15/26 - 10/30/26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Common AACSB Status Values:</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>• Scholarly Academic (SA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>• Practice Academic (PA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>• Scholarly Practitioner (SP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>• Instructional Practitioner (IP)</t>
         </is>

</xml_diff>